<commit_message>
TC-005 to TC-011 and TC-015: Create Slip group passed
Eight cases recorded, all Pass, no new defects found.

Notable evidence:
- TC-009: Tons entered as 36,22 stored as 36.22, comma converted to period
- TC-011: draft re-opened with SlipID 1 and Bill 20260808-103823 unchanged
- TC-005: blocked save left the row count unchanged, and the Bill Number
  generated for the abandoned form was discarded rather than consumed

TC-041 remains open pending the print confirmation, though its critical half is
already proven: the row holds the edited Rom Type and Tons while still Unprinted,
so the DEF-022 fix persisted the edits at Print time as intended.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Case_Matrix.xlsx
+++ b/docs/Test_Case_Matrix.xlsx
@@ -1662,10 +1662,26 @@
       <c r="I6" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="J6" s="3"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Save was blocked with a Validation message reading 'Truck Reg (Field 1) is required before saving.' SlipID remained 'Auto-assigned' and the database row count was unchanged, confirming nothing was written. The Bill Number generated for the abandoned form was discarded rather than consumed, so no gap was created in the sequence.</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -1695,10 +1711,26 @@
       <c r="I7" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="J7" s="3"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>With Truck Reg cleared on an existing saved draft, Print was blocked with 'Truck Reg (Field 1) is required before printing.' - the same strictness applied to Tons.</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
@@ -1728,10 +1760,26 @@
       <c r="I8" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="J8" s="3"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>The slip saved as an Unprinted draft with Tons left blank, and the Main Page tile appeared showing Tons: 0.</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
@@ -1761,10 +1809,26 @@
       <c r="I9" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="J9" s="3"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Print on the draft with Tons still blank was blocked with 'Tons must be filled in before printing.'</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
@@ -1794,10 +1858,26 @@
       <c r="I10" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="J10" s="3"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Tons entered as 36,22 using a comma was stored in the database as 36.22 with a period.</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
@@ -1827,10 +1907,26 @@
       <c r="I11" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="J11" s="3"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>A second decimal separator could not be typed at all - attempting 15.5.3 was refused at the keystroke, so the invalid value never reached the field.</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
@@ -1860,10 +1956,26 @@
       <c r="I12" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="J12" s="3"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Re-opening the draft from its tile showed SlipID 1 and Bill Number 20260808-103823, identical to the values before the edit and re-save. No new identifiers were allocated.</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
@@ -1992,10 +2104,26 @@
       <c r="I16" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="J16" s="3"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Saving a new slip with Truck Reg LFN550NW produced a Main Page tile showing the registration, SlipID and Tons.</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">

</xml_diff>

<commit_message>
Slip Lifecycle group: twelve cases passed, no defects found
TC-016, TC-017, TC-018, TC-019, TC-020, TC-021, TC-022, TC-033, TC-037,
TC-041, TC-042 and TC-043 all recorded Pass.

Key evidence:
- TC-042: slip 1 reprinted twice at 11:18 and 11:20; both previews showed
  'Printed: 2026-08-08 11:13', the original print time, and PrintedAt in the
  database stayed 11:13:58 throughout. The DEF-027 fix and the COALESCE guard
  on MarkSlipAsPrinted both hold.
- TC-041: the draft's edited Rom Type and Tons were in the row while it was
  still Unprinted, proving DEF-022's fix persists at Print time.
- TC-021: voiding a printed slip preserved PrintedAt alongside VoidedAt, so the
  record still shows both that it printed and when it was voided.
- TC-043: Bill Number, CreatedAt, PrintedAt and the date on the paper all agree
  with the machine clock, confirming DEF-026.

26 of 46 cases now executed, all Pass.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Case_Matrix.xlsx
+++ b/docs/Test_Case_Matrix.xlsx
@@ -2153,10 +2153,26 @@
       <c r="I17" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="J17" s="3"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Clicking Print opened the Print Preview before anything reached the printer. No paper was committed until Print was pressed on the preview itself.</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
@@ -2186,10 +2202,26 @@
       <c r="I18" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="J18" s="3"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Confirming the print set slip 1 to Printed with PrintedAt 2026-08-08 11:13:58, removed its Main Page tile, and the slip appeared in Slip History. The daily summary updated to Loads: 1, Total Tons: 36.220 t.</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
@@ -2228,10 +2260,26 @@
           <t>The operator is returned to the same Print Preview, re-rendered with the new settings, rather than being sent to the printer or back to the Main Page.</t>
         </is>
       </c>
-      <c r="J19" s="3"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Opened Calibrate Print from the preview, changed the font scale from 2.35 to 2.55 and saved. The operator was returned to the same Print Preview, re-rendered with the new scale, rather than being sent onward.</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
@@ -2261,10 +2309,26 @@
       <c r="I20" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="J20" s="3"/>
-      <c r="K20" s="6"/>
-      <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Cancel on a saved draft offered Void / Close / Cancel. Confirming with a blank reason was refused with 'A void reason is required.' and the dialog stayed open. After entering a reason the slip voided, its tile disappeared, and it appeared in the Voided view with VoidedAt 2026-08-08 11:25:06.</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
@@ -2294,10 +2358,26 @@
       <c r="I21" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="J21" s="3"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>The reason field stopped accepting input at exactly 20 characters. Confirmed on both void dialogs - the one reached from Cancel on a draft, and the one reached from Void Slip on a printed slip. Stored values measured 20 and 6 characters.</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
@@ -2327,10 +2407,26 @@
       <c r="I22" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="J22" s="3"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Slip 1, already Printed, was voided from Slip History with a reason. A blank reason was refused first. The slip moved to Voided with VoidedAt 2026-08-08 11:33:20 while PrintedAt was preserved at 11:13:58, so the record still shows both that it was printed and when it was voided. Nothing was deleted.</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
@@ -2360,10 +2456,26 @@
       <c r="I23" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="J23" s="3"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Slip 1 was reprinted twice from Slip History, at 11:18 and 11:20, with no restriction, warning or error on either attempt.</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
@@ -2723,10 +2835,26 @@
       <c r="I34" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="J34" s="3"/>
-      <c r="K34" s="6"/>
-      <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>The Printed view showed only Printed slips and the Voided view only Voided ones. The Voided view additionally showed the Void Reason and Voided At columns, both populated, and those columns were absent from the Printed view.</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
@@ -2876,10 +3004,26 @@
       <c r="I38" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="J38" s="3"/>
-      <c r="K38" s="6"/>
-      <c r="L38" s="3"/>
-      <c r="M38" s="3"/>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>With the only slip printed and its tile removed, the Main Page showed 'Welcome! Your slips will appear here. Click New Slip to get started.' instead of an empty panel.</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
@@ -3030,10 +3174,26 @@
           <t>The edited values are written to the database before printing, so the printed slip and its stored row are identical. No printed slip may ever disagree with its database record.</t>
         </is>
       </c>
-      <c r="J42" s="3"/>
-      <c r="K42" s="6"/>
-      <c r="L42" s="3"/>
-      <c r="M42" s="3"/>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Rom Type and Tons were edited on a saved draft and Print was clicked without Save. The database row held the edited values (MG2/3W and 36.22) while still Unprinted, proving the edits were persisted at Print time; the preview and the printed slip carried the same values, and Slip History confirmed them after the print completed.</t>
+        </is>
+      </c>
+      <c r="K42" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="inlineStr">
@@ -3084,10 +3244,26 @@
           <t>The preview shows the slip's ORIGINAL print date, not today's. Printed At is unchanged afterwards and the slip holds its position in the history ordering.</t>
         </is>
       </c>
-      <c r="J43" s="3"/>
-      <c r="K43" s="6"/>
-      <c r="L43" s="3"/>
-      <c r="M43" s="3"/>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Slip 1 was reprinted twice at 11:18 and 11:20. Both previews showed 'Printed: 2026-08-08 11:13' - the original print time, not the time of the reprint - and PrintedAt in the database remained 11:13:58 throughout, so the slip kept its position in the history ordering.</t>
+        </is>
+      </c>
+      <c r="K43" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="inlineStr">
@@ -3137,10 +3313,26 @@
           <t>All four agree with the PC clock. None is offset by the machine's UTC difference. The same holds on any machine the application is installed on.</t>
         </is>
       </c>
-      <c r="J44" s="3"/>
-      <c r="K44" s="6"/>
-      <c r="L44" s="3"/>
-      <c r="M44" s="3"/>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>All four sources agreed with the PC clock, with no UTC offset. Slip 1: Bill Number 20260808-103823 (10:38:23), CreatedAt 10:41:10, PrintedAt 11:13:58, and the date printed on the slip read 2026-08-08 11:13. The same held for slips 2 and 3.</t>
+        </is>
+      </c>
+      <c r="K44" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Data Integrity group: TC-012, TC-013, TC-014 and TC-031 passed
The three immutability guarantees are confirmed end to end.

TC-012 - SlipID is read-only on every screen that shows it, and a printed slip
cannot be opened in Create Slip at all, so no path exposes it as editable.
TC-013 - Bill Number is absent from the History Edit tab entirely and read-only
on Create Slip, with the PreventBillNumberChange trigger backing it at the
storage layer.
TC-014 - slip 4 took Bill 20260811-082225, was voided, and the next slip opened
with 20260811-082426. The consumed number was never reissued.
TC-031 - selecting a grid row populated the Edit tab with the correct slip.

38 of 46 cases executed, all Pass.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Case_Matrix.xlsx
+++ b/docs/Test_Case_Matrix.xlsx
@@ -2005,10 +2005,26 @@
       <c r="I13" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="J13" s="3"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>On the Slip History Edit tab the Slip ID showed 3 in a greyed, uneditable box. On Create Slip the field read 'Auto-assigned' before saving and 4 afterwards, read-only in both states. A printed slip cannot be opened in Create Slip at all - editing a printed slip is done through the History Edit tab by design - so there is no screen anywhere that exposes SlipID as editable.</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
@@ -2038,10 +2054,26 @@
       <c r="I14" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="J14" s="3"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Bill Number is absent from the Slip History Edit tab entirely, so there is no control through which to change it. On Create Slip it is displayed read-only. The database additionally rejects any UPDATE to the column through the PreventBillNumberChange trigger, giving protection at both the UI and storage layers.</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
@@ -2071,10 +2103,26 @@
       <c r="I15" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="J15" s="3"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Slip 4 was created with Bill Number 20260811-082225 and then voided at 08:24:24 with reason 'Test'. The next new slip opened with Bill Number 20260811-082426 - a different and later value. The voided slip retained its own number and it was never reissued.</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
@@ -2833,10 +2881,26 @@
       <c r="I32" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="J32" s="3"/>
-      <c r="K32" s="6"/>
-      <c r="L32" s="3"/>
-      <c r="M32" s="3"/>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Selecting slip 3 in the grid populated the Edit Slip tab with that slip's details: Slip ID 3, Truck Reg LFN550NW, Stockpile Name MSMG2/3W, Rom Type MG2/3W, Block Nr BL7, Size -40, Slot number ACACIA and Tons 36.98. Every field was editable except Slip ID, and Bill Number was not present.</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">

</xml_diff>

<commit_message>
Printer Settings and Slip History mechanics: TC-027, TC-028, TC-030, TC-032 passed
TC-028 confirms DEF-008 at runtime. A second preset was saved to repeatedly,
including a font scale change from 2.60 to 1.60, and the database still holds
exactly two profiles with the latest values on the edited one. The
ON CONFLICT(ProfileName) DO UPDATE upsert behaves as an in-place update.

TC-027 also showed the selection becoming the active profile and GlobalSettings
syncing to it.

42 of 46 executed, all Pass. Remaining: TC-029 (known failure, calibration grid
has no caller), TC-038, TC-039, TC-040.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Case_Matrix.xlsx
+++ b/docs/Test_Case_Matrix.xlsx
@@ -2749,10 +2749,26 @@
       <c r="I28" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="J28" s="3"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>A second preset named 'TC-27 test' was created with paper Small151x151 and 2 copies, alongside the existing 'Default' at A4 with 1 copy. Switching the dropdown between them changed the form values to match each preset, and the selection also became the active profile in the database: TC-27 test IsActive=1, Default IsActive=0. GlobalSettings synced to the active preset's paper size and copy count.</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
@@ -2782,10 +2798,26 @@
       <c r="I29" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="J29" s="3"/>
-      <c r="K29" s="6"/>
-      <c r="L29" s="3"/>
-      <c r="M29" s="3"/>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Calibration and configuration were saved to 'TC-27 test' several times, including a font scale change from 2.60 to 1.60. The database afterwards held exactly two profiles, Default and TC-27 test, with no duplicate entry, and TC-27 test carried the latest values. This confirms the ON CONFLICT(ProfileName) DO UPDATE upsert behaviour recorded under DEF-008.</t>
+        </is>
+      </c>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
@@ -2848,10 +2880,26 @@
       <c r="I31" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="J31" s="3"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="3"/>
-      <c r="M31" s="3"/>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Clicking directly into any cell of the Slip History grid did not enter an editable state and no text could be typed.</t>
+        </is>
+      </c>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
@@ -2930,10 +2978,26 @@
       <c r="I33" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="J33" s="3"/>
-      <c r="K33" s="6"/>
-      <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Setting the date range to 8 August returned no rows; 10 August returned slip 3; a range spanning both returned slip 3. Only slips falling inside the selected range were shown.</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">

</xml_diff>

<commit_message>
Main Page and Backup group: TC-038, TC-039, TC-040 passed
45 of 46 executed. TC-029 is the only case not yet run.

TC-039 doubles as clean before/after evidence for DEF-018: every backup taken
since the fix has a Date modified matching its filename timestamp, while the
older pre-fix files still show the mismatch, e.g. WeighbridgeData_20260805_080052
stamped 14 July.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Case_Matrix.xlsx
+++ b/docs/Test_Case_Matrix.xlsx
@@ -3293,10 +3293,26 @@
       <c r="I39" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="J39" s="3"/>
-      <c r="K39" s="6"/>
-      <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>33 unprinted drafts were created. Beyond roughly 28 tiles the panel became scrollable, a scrollbar appeared on the right, and every tile from slip 5 through slip 33 remained reachable by scrolling. No tiles were clipped or lost off-screen.</t>
+        </is>
+      </c>
+      <c r="K39" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
@@ -3326,10 +3342,26 @@
       <c r="I40" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="J40" s="3"/>
-      <c r="K40" s="6"/>
-      <c r="L40" s="3"/>
-      <c r="M40" s="3"/>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>The Backups folder held a file named WeighbridgeData_20260811_082055.db stamped 8/11/2026 8:20 AM, created by that morning's launch. Every backup taken since the DEF-018 fix carries a Date modified matching its filename timestamp, while the older pre-fix files still show the mismatch that defect described - for example WeighbridgeData_20260805_080052.db stamped 14 July.</t>
+        </is>
+      </c>
+      <c r="K40" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
@@ -3359,10 +3391,26 @@
       <c r="I41" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="J41" s="3"/>
-      <c r="K41" s="6"/>
-      <c r="L41" s="3"/>
-      <c r="M41" s="3"/>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Backup Now opened a Save Database Backup dialog defaulting to a .db filename. A destination outside the application folder was chosen and the file saved, with a Backup Complete message confirming the full path it was written to.</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="inlineStr">

</xml_diff>